<commit_message>
Add double precision to read cbb budget files
</commit_message>
<xml_diff>
--- a/assets/3D/setup.xlsx
+++ b/assets/3D/setup.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\assets\3D\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{048CD627-3D18-4419-9C58-1E37C295613E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA972E6-B9AB-41A2-91E4-5FC98C80BD76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17247,7 +17247,7 @@
         <v>300</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I2">
         <v>70</v>
@@ -17316,8 +17316,8 @@
       <c r="G4">
         <v>150</v>
       </c>
-      <c r="H4">
-        <v>3</v>
+      <c r="H4" s="4">
+        <v>5</v>
       </c>
       <c r="I4">
         <v>70</v>
@@ -17351,7 +17351,7 @@
       <c r="G5">
         <v>100</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="4">
         <v>5</v>
       </c>
       <c r="I5">
@@ -17386,8 +17386,8 @@
       <c r="G6">
         <v>0</v>
       </c>
-      <c r="H6">
-        <v>3</v>
+      <c r="H6" s="4">
+        <v>5</v>
       </c>
       <c r="I6">
         <v>70</v>

</xml_diff>